<commit_message>
Añade trazabilidad SHA-256 a fuentes y exportaciones
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
+++ b/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
@@ -11,9 +11,13 @@
     <sheet name="Escala por correlacion" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Detalle Plantilla 87" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Metodologia y fuentes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Trazabilidad SHA-256" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle Plantilla 87'!$A$1:$E$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trazabilidad SHA-256'!$A$6:$G$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Trazabilidad SHA-256'!$1:$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Trazabilidad SHA-256'!$A$1:$G$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +30,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,8 +86,34 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00536875"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -125,8 +155,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF0F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5EE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -148,11 +188,16 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="hair">
+        <color rgb="00CBD5DC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -256,6 +301,26 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -330,6 +395,22 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifiestoSHA256" displayName="ManifiestoSHA256" ref="A6:G12" headerRowCount="1">
+  <autoFilter ref="A6:G12"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Fuente"/>
+    <tableColumn id="3" name="Ruta del repositorio"/>
+    <tableColumn id="4" name="Estado"/>
+    <tableColumn id="5" name="SHA-256 aprobado"/>
+    <tableColumn id="6" name="SHA-256 actual"/>
+    <tableColumn id="7" name="Tamaño (bytes)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6907,4 +6988,339 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="76" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="68" customWidth="1" min="5" max="5"/>
+    <col width="68" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>TRAZABILIDAD DE FUENTES · CAPITAL HUMANO</t>
+        </is>
+      </c>
+      <c r="B1" s="35" t="n"/>
+      <c r="C1" s="35" t="n"/>
+      <c r="D1" s="35" t="n"/>
+      <c r="E1" s="35" t="n"/>
+      <c r="F1" s="35" t="n"/>
+      <c r="G1" s="35" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>Versión de la aplicación</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.1.0-dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="36" t="inlineStr">
+        <is>
+          <t>Integridad del manifiesto</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="36" t="inlineStr">
+        <is>
+          <t>Verificación UTC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-28T21:19:21+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>SHA-256 compara los bytes con el manifiesto versionado; no sustituye revisión normativa ni firma digital.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="38" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>Ruta del repositorio</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>SHA-256 aprobado</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>SHA-256 actual</t>
+        </is>
+      </c>
+      <c r="G6" s="38" t="inlineStr">
+        <is>
+          <t>Tamaño (bytes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>plantilla_res87</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Plantilla de cargos · propuesta Resolución 87</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>Nueva Estructura de Plantilla/Organigrama/propuesta de plantilla por la resolucion 87.xls</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>02399d1abf33cb821829df57f146e9011488ed86a11e539c664a2114c7b8b6cc</t>
+        </is>
+      </c>
+      <c r="F7" s="42" t="inlineStr">
+        <is>
+          <t>02399d1abf33cb821829df57f146e9011488ed86a11e539c664a2114c7b8b6cc</t>
+        </is>
+      </c>
+      <c r="G7" s="39" t="n">
+        <v>2780672</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="39" t="inlineStr">
+        <is>
+          <t>escala_res29</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>Escala histórica · Resolución 29/2020</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>TES/Salariales/Escala 3210_OK.xlsx</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+      <c r="E8" s="42" t="inlineStr">
+        <is>
+          <t>fbf1764dd6d77a5845dbbd01a7453e119915feb798dc7b43f25e431f67217d01</t>
+        </is>
+      </c>
+      <c r="F8" s="42" t="inlineStr">
+        <is>
+          <t>fbf1764dd6d77a5845dbbd01a7453e119915feb798dc7b43f25e431f67217d01</t>
+        </is>
+      </c>
+      <c r="G8" s="39" t="n">
+        <v>13968</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="39" t="inlineStr">
+        <is>
+          <t>gaceta_2026</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>Gaceta Oficial · Resoluciones 14/2026 y 15/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>TES/Salariales/goc-2026-o60.pdf</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>7dfe261ae1db5de5ceee1e9ebe141693a5a1ca474809158960c6bd94a2c0a1e1</t>
+        </is>
+      </c>
+      <c r="F9" s="42" t="inlineStr">
+        <is>
+          <t>7dfe261ae1db5de5ceee1e9ebe141693a5a1ca474809158960c6bd94a2c0a1e1</t>
+        </is>
+      </c>
+      <c r="G9" s="39" t="n">
+        <v>1104320</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="39" t="inlineStr">
+        <is>
+          <t>motor_calculo</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Código de extracción y cálculo</t>
+        </is>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>TES/Salariales/Nueva Escala 3210/generar_escala.py</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>c41ad5dfcdabc308705d391cca7309377ba1dd7ec855c06bfe49b28a32c272e8</t>
+        </is>
+      </c>
+      <c r="F10" s="42" t="inlineStr">
+        <is>
+          <t>c41ad5dfcdabc308705d391cca7309377ba1dd7ec855c06bfe49b28a32c272e8</t>
+        </is>
+      </c>
+      <c r="G10" s="39" t="n">
+        <v>37562</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>interfaz_app</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>Código de la aplicación y exportadores</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>TES/Salariales/Nueva Escala 3210/app_escala.py</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>710421e5c5d23bf9ab5626b37c60f164720012678a82454c98fad5aa0ac900cb</t>
+        </is>
+      </c>
+      <c r="F11" s="42" t="inlineStr">
+        <is>
+          <t>710421e5c5d23bf9ab5626b37c60f164720012678a82454c98fad5aa0ac900cb</t>
+        </is>
+      </c>
+      <c r="G11" s="39" t="n">
+        <v>39479</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>actualizador_manifest</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t>Herramienta de actualización del manifiesto</t>
+        </is>
+      </c>
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>tools/actualizar_manifiesto_fuentes.py</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+      <c r="E12" s="42" t="inlineStr">
+        <is>
+          <t>6b820ded8d9c01129c0d5fbfa223e43039be6126db75809c15d5ea675f2c5e85</t>
+        </is>
+      </c>
+      <c r="F12" s="42" t="inlineStr">
+        <is>
+          <t>6b820ded8d9c01129c0d5fbfa223e43039be6126db75809c15d5ea675f2c5e85</t>
+        </is>
+      </c>
+      <c r="G12" s="39" t="n">
+        <v>865</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G12"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="2"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Carga el motor salarial desde la ruta de la aplicación
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
+++ b/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
@@ -7053,7 +7053,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-28T21:19:21+00:00</t>
+          <t>2026-10-28T21:28:01+00:00</t>
         </is>
       </c>
     </row>
@@ -7264,16 +7264,16 @@
       </c>
       <c r="E11" s="42" t="inlineStr">
         <is>
-          <t>710421e5c5d23bf9ab5626b37c60f164720012678a82454c98fad5aa0ac900cb</t>
+          <t>a23da7c8ab2f8da01dc68cdadb8509874137c86b8fb1b8ad7f7587b591a6edae</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
-          <t>710421e5c5d23bf9ab5626b37c60f164720012678a82454c98fad5aa0ac900cb</t>
+          <t>a23da7c8ab2f8da01dc68cdadb8509874137c86b8fb1b8ad7f7587b591a6edae</t>
         </is>
       </c>
       <c r="G11" s="39" t="n">
-        <v>39479</v>
+        <v>40079</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Añade informe imprimible de metodología y aprobación
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
+++ b/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
@@ -7053,7 +7053,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-28T21:28:01+00:00</t>
+          <t>2026-10-28T22:03:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7264,16 +7264,16 @@
       </c>
       <c r="E11" s="42" t="inlineStr">
         <is>
-          <t>a23da7c8ab2f8da01dc68cdadb8509874137c86b8fb1b8ad7f7587b591a6edae</t>
+          <t>ee25477b30fad036b861ebc1f46f21922de217576a95200ed27b836a0d6421de</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
-          <t>a23da7c8ab2f8da01dc68cdadb8509874137c86b8fb1b8ad7f7587b591a6edae</t>
+          <t>ee25477b30fad036b861ebc1f46f21922de217576a95200ed27b836a0d6421de</t>
         </is>
       </c>
       <c r="G11" s="39" t="n">
-        <v>40079</v>
+        <v>51698</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Añade diagnóstico de calidad de la plantilla
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
+++ b/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
@@ -7608,7 +7608,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:18:57+00:00</t>
+          <t>2026-10-28T22:40:37+00:00</t>
         </is>
       </c>
     </row>
@@ -7784,16 +7784,16 @@
       </c>
       <c r="E10" s="42" t="inlineStr">
         <is>
-          <t>259b3e28b7d715fe7fb2cd0eaea0f440fd0df3a48199cf306ba89c5902f42d9b</t>
+          <t>7ab5a4346d21ac5bb85389c006f81741a9afc03ea4f3058cf17ab24ea2f45a13</t>
         </is>
       </c>
       <c r="F10" s="42" t="inlineStr">
         <is>
-          <t>259b3e28b7d715fe7fb2cd0eaea0f440fd0df3a48199cf306ba89c5902f42d9b</t>
+          <t>7ab5a4346d21ac5bb85389c006f81741a9afc03ea4f3058cf17ab24ea2f45a13</t>
         </is>
       </c>
       <c r="G10" s="39" t="n">
-        <v>38904</v>
+        <v>43005</v>
       </c>
     </row>
     <row r="11">
@@ -7819,16 +7819,16 @@
       </c>
       <c r="E11" s="42" t="inlineStr">
         <is>
-          <t>d3d445fe400ce174942b4dad8f2ff5b1d96d05e0a53580b851a8428439aea6e7</t>
+          <t>b0a794ad3c4c6e5e6c204d808480d50725c2afd2b471808f32dde14d51940515</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
-          <t>d3d445fe400ce174942b4dad8f2ff5b1d96d05e0a53580b851a8428439aea6e7</t>
+          <t>b0a794ad3c4c6e5e6c204d808480d50725c2afd2b471808f32dde14d51940515</t>
         </is>
       </c>
       <c r="G11" s="39" t="n">
-        <v>54531</v>
+        <v>56412</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Evita superposición del pie en el PDF de plantilla
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
+++ b/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
@@ -7608,7 +7608,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:40:37+00:00</t>
+          <t>2026-10-28T22:47:29+00:00</t>
         </is>
       </c>
     </row>
@@ -7819,16 +7819,16 @@
       </c>
       <c r="E11" s="42" t="inlineStr">
         <is>
-          <t>b0a794ad3c4c6e5e6c204d808480d50725c2afd2b471808f32dde14d51940515</t>
+          <t>247abb24916ab26d432365a991e389986e62dff1e658156c817145354cd84b03</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
-          <t>b0a794ad3c4c6e5e6c204d808480d50725c2afd2b471808f32dde14d51940515</t>
+          <t>247abb24916ab26d432365a991e389986e62dff1e658156c817145354cd84b03</t>
         </is>
       </c>
       <c r="G11" s="39" t="n">
-        <v>56412</v>
+        <v>56637</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Resolve authorized salary group discrepancies
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
+++ b/TES/Salariales/Nueva Escala 3210/Escala_Salarial_3210_Nueva.xlsx
@@ -15,9 +15,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle Plantilla 87'!$A$1:$F$184</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trazabilidad SHA-256'!$A$6:$G$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trazabilidad SHA-256'!$A$6:$G$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Trazabilidad SHA-256'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Trazabilidad SHA-256'!$A$1:$G$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Trazabilidad SHA-256'!$A$1:$G$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -398,8 +398,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifiestoSHA256" displayName="ManifiestoSHA256" ref="A6:G12" headerRowCount="1">
-  <autoFilter ref="A6:G12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifiestoSHA256" displayName="ManifiestoSHA256" ref="A6:G13" headerRowCount="1">
+  <autoFilter ref="A6:G13"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Fuente"/>
@@ -726,7 +726,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado el 28/10/2026. La columna G se alimenta del archivo “propuesta de plantilla por la resolucion 87.xls”. Montos en pesos cubanos (CUP).</t>
+          <t>Generado el 29/10/2026. La columna G se alimenta del archivo “propuesta de plantilla por la resolucion 87.xls”. Montos en pesos cubanos (CUP).</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
         <is>
-          <t>NOTAS: Grupo XII: valores encontrados -&gt; $5,770.00 (15 ocurrencias), $5,570.00 (1 ocurrencias). Se adopta $5,770.00 por ser el mayoritario. / Grupo XV: valores encontrados -&gt; $7,201.00 (5 ocurrencias), $7,777.00 (1 ocurrencias). Se adopta $7,201.00 por ser el mayoritario.</t>
+          <t>NOTAS: sin anomalías.</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="F28" s="28" t="n">
-        <v>7777</v>
+        <v>7201</v>
       </c>
     </row>
     <row r="29">
@@ -5197,7 +5197,7 @@
         </is>
       </c>
       <c r="F98" s="28" t="n">
-        <v>5570</v>
+        <v>5770</v>
       </c>
     </row>
     <row r="99">
@@ -7448,7 +7448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -7516,25 +7516,11 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="34" t="inlineStr">
-        <is>
-          <t>• Grupo XII: valores encontrados -&gt; $5,770.00 (15 ocurrencias), $5,570.00 (1 ocurrencias). Se adopta $5,770.00 por ser el mayoritario.</t>
-        </is>
-      </c>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="34" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="34" t="inlineStr">
-        <is>
-          <t>• Grupo XV: valores encontrados -&gt; $7,201.00 (5 ocurrencias), $7,777.00 (1 ocurrencias). Se adopta $7,201.00 por ser el mayoritario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="34" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="34" t="inlineStr">
         <is>
           <t>LENGUAJE DE PROGRAMACIÓN UTILIZADO: Python 3 — librerías xlrd (lectura del .xls heredado), openpyxl (Excel con fórmulas/estilos) y fpdf2 (PDF). Es la opción más adecuada porque lee formatos legacy, permite auditoría registro a registro, se re-ejecuta sin intervención manual y genera ambos formatos de salida con un único código mantenible.</t>
         </is>
@@ -7551,7 +7537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7608,7 +7594,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:47:29+00:00</t>
+          <t>2026-10-29T00:52:01+00:00</t>
         </is>
       </c>
     </row>
@@ -7679,12 +7665,12 @@
       </c>
       <c r="E7" s="42" t="inlineStr">
         <is>
-          <t>02399d1abf33cb821829df57f146e9011488ed86a11e539c664a2114c7b8b6cc</t>
+          <t>5542e23b705462738e66a82ed1aec8d60727c6d1352438266e620878ab63e473</t>
         </is>
       </c>
       <c r="F7" s="42" t="inlineStr">
         <is>
-          <t>02399d1abf33cb821829df57f146e9011488ed86a11e539c664a2114c7b8b6cc</t>
+          <t>5542e23b705462738e66a82ed1aec8d60727c6d1352438266e620878ab63e473</t>
         </is>
       </c>
       <c r="G7" s="39" t="n">
@@ -7784,16 +7770,16 @@
       </c>
       <c r="E10" s="42" t="inlineStr">
         <is>
-          <t>7ab5a4346d21ac5bb85389c006f81741a9afc03ea4f3058cf17ab24ea2f45a13</t>
+          <t>11da9e812e996110373df74759d9eb17c49a7fce58fa00e5d7c4c24b1d05adbf</t>
         </is>
       </c>
       <c r="F10" s="42" t="inlineStr">
         <is>
-          <t>7ab5a4346d21ac5bb85389c006f81741a9afc03ea4f3058cf17ab24ea2f45a13</t>
+          <t>11da9e812e996110373df74759d9eb17c49a7fce58fa00e5d7c4c24b1d05adbf</t>
         </is>
       </c>
       <c r="G10" s="39" t="n">
-        <v>43005</v>
+        <v>43127</v>
       </c>
     </row>
     <row r="11">
@@ -7819,16 +7805,16 @@
       </c>
       <c r="E11" s="42" t="inlineStr">
         <is>
-          <t>247abb24916ab26d432365a991e389986e62dff1e658156c817145354cd84b03</t>
+          <t>749b33588504192a5ccf2d062bcb689e7498f75547c355918252216bcec97ef1</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
-          <t>247abb24916ab26d432365a991e389986e62dff1e658156c817145354cd84b03</t>
+          <t>749b33588504192a5ccf2d062bcb689e7498f75547c355918252216bcec97ef1</t>
         </is>
       </c>
       <c r="G11" s="39" t="n">
-        <v>56637</v>
+        <v>75282</v>
       </c>
     </row>
     <row r="12">
@@ -7866,8 +7852,43 @@
         <v>865</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>verificador_paquete</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>Verificador offline de paquetes de exportación</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="inlineStr">
+        <is>
+          <t>tools/verificar_paquete_exportacion.py</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>VERIFICADA</t>
+        </is>
+      </c>
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>0633c843d086b003c6ebaffafdd2c88abd2b463bcf912c80c0ba9a607ec5cbdb</t>
+        </is>
+      </c>
+      <c r="F13" s="42" t="inlineStr">
+        <is>
+          <t>0633c843d086b003c6ebaffafdd2c88abd2b463bcf912c80c0ba9a607ec5cbdb</t>
+        </is>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>8341</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:G12"/>
+  <autoFilter ref="A6:G13"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>

</xml_diff>